<commit_message>
Correct the capability workbook's claim about spatial chunking
The workbook said chunking exists but is unsafe without halo buffering.
It does not exist. The agent layer batches features by vertex weight to
keep memory bounded, which is a batching strategy and not a spatial
tiling, and it does not preserve topology across batches. A reader
checking the claim would look for a chunking module and find none.

The area is now recorded as not built, with what a correct implementation
would have to do: buffer each tile by a halo so a feature crossing a
boundary is present on both sides, and keep whole-layer union and degree
checks in a single global pass because they cannot be tiled.

Five built areas were also missing from the sheet entirely: cloud-
optimized GeoTIFF, OSM data, vertical datum, hardware feasibility and the
governance gates. All are implemented and registered; the sheet simply
had not caught up. It now lists 34 areas, 27 of them built.
</commit_message>
<xml_diff>
--- a/docs/geoqa_capability_matrix.xlsx
+++ b/docs/geoqa_capability_matrix.xlsx
@@ -16,7 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Coverage'!$A$1:$E$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Coverage'!$A$1:$E$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Problem registry'!$A$1:$J$254</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Validator functions'!$A$1:$E$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Profiles'!$A$1:$D$13</definedName>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14">
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -798,7 +798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1263,53 +1263,53 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Spatial chunking</t>
+          <t>Cloud-optimized GeoTIFF</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>built</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Chunking exists but is unsafe for global topology without halo buffering.</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Naive chunking splits connectivity. Halo-buffered chunks required; whole-layer union checks may need a single global pass.</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
+          <t>4 conditions: cloud-optimized layout, missing or undersized overviews, tile size against the declared block size, and whether the format is marked as standing rather than transitional.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Layout only. It reads structure, not pixels; band content validation is the raster adapter's job.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Conflict resolution</t>
+          <t>OSM data</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>not built</t>
+          <t>built</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>No collapsing of competing source records onto one logical feature.</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Numbered key selection with uniqueness evidence and declared precedence, retaining original values rather than overwriting them.</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
+          <t>5 conditions: licence and attribution declaration, version and timestamp metadata, and geometry emergent from unconnected ways rather than authored as features.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>The point is that OSM geometry is assembled from relations at render time. A validator that assumes a closed polygon is testing the extractor's behaviour rather than the data's.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Archive and package inspection</t>
+          <t>Vertical datum</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1319,20 +1319,16 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>13 conditions: zip-slip traversal, absolute paths, unsafe names, decompression bombs, total size, encryption, duplicate members, content-versus-extension mismatch, unreadable members, incomplete shapefile sets, missing CRS sidecars, nested archives, and archives with no geospatial content</t>
+          <t>7 conditions: declared reference surface, depth sign convention, missing vertical component on data that requires one, compound CRS requirements, and unit reasoning on vertical attributes.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Inspects without extracting. Member names are checked for traversal and content is checked against magic bytes, because a .shp containing XML will not open and a .shp containing a ZIP is a real occurrence. Verified against 41 archives in a real downloads folder.</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Tabular sources</t>
+          <t>Hardware feasibility</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1342,20 +1338,20 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>17 conditions: missing and duplicate headers, ragged rows, identifier leading-zero loss, over-long numeric identifiers, ambiguous day/month dates, instrument sentinels, merged cells, hidden sheets and rows, formulas, empty columns, missing keys and duplicate keys</t>
+          <t>CPU temperature and throttling headroom, available memory against the estimated working set, free disk against the projected output, and GPU presence where a step needs one.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Targets the failures that produce plausible wrong data rather than errors. Excel turns 007123 into 7123 and 03/04 into a different month; both survive every downstream check.</t>
+          <t>Reports whether this machine can carry out the operation before it is attempted, so a long run stops on evidence rather than on the operator noticing a hot laptop.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Coordinate axis order</t>
+          <t>Governance gates</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1365,66 +1361,66 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>6 conditions: undeclared order, swapped axes, ambiguous order, outside extent, non-numeric coordinates, and declaration versus column-name conflict. SQL generators for PostgreSQL and PostGIS are provided and return the query rather than taking a connection.</t>
+          <t>Declared release gates that evaluate findings, record which issues triggered them, and hold for a named human decision. llm_involved is a class constant rather than a setting, so a gate cannot be constructed that claims not to consult a model while doing so.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>EPSG:4326 is formally latitude/longitude while GeoJSON, PostGIS and desktop GIS are longitude/latitude. Both readings of an in-range pair are legal, so an ambiguous pair is reported as evidence and needs a declared extent to become a verdict.</t>
+          <t>Recall is scored against expected outcomes rather than remembered, so the hit rate is a number the library produces. Each property is covered by a test that fails if it stops being true.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Credential and disclosure safety</t>
+          <t>Spatial chunking</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>built</t>
+          <t>not built</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Provider-prefixed token patterns, PEM private key blocks, connection strings with inline passwords, URL basic auth, and entropy-gated secret-named literals; plus 5 conditions for credentials, blocked terms, sensitive columns, personal data and filesystem paths that would be sent to a model</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Detection has explicit exemptions for environment references, placeholders and short values, because a detector that cries wolf is switched off and then protects nothing.</t>
-        </is>
-      </c>
+          <t>No spatial chunking exists. The agent layer batches features by vertex weight to keep memory bounded; that is a batching strategy, not a spatial tiling, and it does not preserve topology across batches.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>A tiled implementation must buffer each tile by a halo so a feature crossing a boundary is present on both sides, otherwise connectivity checks report false breaks at the seams. Whole-layer union and degree checks cannot be tiled at all and need a single global pass. Until both exist, any large-layer run must complete in one pass.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Clipping conformance</t>
+          <t>Conflict resolution</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>built</t>
+          <t>not built</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>8 conditions: straddling evidence with a measured split, assignment near the threshold, unresolved assignment, half-area features, heavily truncated features, features missing after a clip, clipped features with no source, and the evidence condition itself</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>The assignment percentage is a caller-supplied parameter, not a constant, because it is an organisational policy. Half-geometry is detected by area ratio against the source, which catches a centreline clip that no validity check would.</t>
-        </is>
-      </c>
+          <t>No collapsing of competing source records onto one logical feature.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Numbered key selection with uniqueness evidence and declared precedence, retaining original values rather than overwriting them.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Workbook attachments</t>
+          <t>Archive and package inspection</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1434,20 +1430,20 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>9 conditions: broken path references, orphaned attachments, duplicate content, attachments below a legibility threshold, undecodable formats, unattributable rows, rows missing an attachment, unverifiable keys, and a workbook with no media at all</t>
+          <t>13 conditions: zip-slip traversal, absolute paths, unsafe names, decompression bombs, total size, encryption, duplicate members, content-versus-extension mismatch, unreadable members, incomplete shapefile sets, missing CRS sidecars, nested archives, and archives with no geospatial content</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Domain-neutral by construction: the artefact is called an attachment and the row a record, so the same checks serve any evidence-per-row workflow.</t>
+          <t>Inspects without extracting. Member names are checked for traversal and content is checked against magic bytes, because a .shp containing XML will not open and a .shp containing a ZIP is a real occurrence. Verified against 41 archives in a real downloads folder.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Metadata governance</t>
+          <t>Tabular sources</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1457,41 +1453,156 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>11 conditions: undeclared licence, non-open licence, unassigned accountability, undeclared lineage, undeclared conformity, missing unique identifier, missing temporal reference, stale metadata, and missing or placeholder elements</t>
+          <t>17 conditions: missing and duplicate headers, ragged rows, identifier leading-zero loss, over-long numeric identifiers, ambiguous day/month dates, instrument sentinels, merged cells, hidden sheets and rows, formulas, empty columns, missing keys and duplicate keys</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Required elements and multiplicities follow Commission Regulation (EC) No 1205/2008; open-by-default follows Directive (EU) 2019/1024. Chosen as a citable checklist because it specifies multiplicities, which makes missing decidable rather than a matter of taste.</t>
+          <t>Targets the failures that produce plausible wrong data rather than errors. Excel turns 007123 into 7123 and 03/04 into a different month; both survive every downstream check.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>Coordinate axis order</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>6 conditions: undeclared order, swapped axes, ambiguous order, outside extent, non-numeric coordinates, and declaration versus column-name conflict. SQL generators for PostgreSQL and PostGIS are provided and return the query rather than taking a connection.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>EPSG:4326 is formally latitude/longitude while GeoJSON, PostGIS and desktop GIS are longitude/latitude. Both readings of an in-range pair are legal, so an ambiguous pair is reported as evidence and needs a declared extent to become a verdict.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Credential and disclosure safety</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Provider-prefixed token patterns, PEM private key blocks, connection strings with inline passwords, URL basic auth, and entropy-gated secret-named literals; plus 5 conditions for credentials, blocked terms, sensitive columns, personal data and filesystem paths that would be sent to a model</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Detection has explicit exemptions for environment references, placeholders and short values, because a detector that cries wolf is switched off and then protects nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Clipping conformance</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>8 conditions: straddling evidence with a measured split, assignment near the threshold, unresolved assignment, half-area features, heavily truncated features, features missing after a clip, clipped features with no source, and the evidence condition itself</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>The assignment percentage is a caller-supplied parameter, not a constant, because it is an organisational policy. Half-geometry is detected by area ratio against the source, which catches a centreline clip that no validity check would.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Workbook attachments</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>9 conditions: broken path references, orphaned attachments, duplicate content, attachments below a legibility threshold, undecodable formats, unattributable rows, rows missing an attachment, unverifiable keys, and a workbook with no media at all</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Domain-neutral by construction: the artefact is called an attachment and the row a record, so the same checks serve any evidence-per-row workflow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Metadata governance</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>built</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>11 conditions: undeclared licence, non-open licence, unassigned accountability, undeclared lineage, undeclared conformity, missing unique identifier, missing temporal reference, stale metadata, and missing or placeholder elements</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Required elements and multiplicities follow Commission Regulation (EC) No 1205/2008; open-by-default follows Directive (EU) 2019/1024. Chosen as a citable checklist because it specifies multiplicities, which makes missing decidable rather than a matter of taste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Packaging and distribution</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>blocked</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>PyPI name geoqa is taken by an unrelated package; GitHub has a functional QGIS-plugin collision.</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Resolve naming before public release. Repository name can stay.</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E30"/>
+  <autoFilter ref="A1:E35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Regenerate the capability workbook with chunking recorded as built
Spatial chunking moves from not built to partial. It is partial rather than
built because the tiling is not yet wired into the runtime dispatch, and
the budget is a vertex count rather than a measured memory ceiling. Both
are recorded in the gap column rather than left for a reader to discover.
</commit_message>
<xml_diff>
--- a/docs/geoqa_capability_matrix.xlsx
+++ b/docs/geoqa_capability_matrix.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Coverage'!$A$1:$E$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Problem registry'!$A$1:$J$254</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Problem registry'!$A$1:$J$256</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Validator functions'!$A$1:$E$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Profiles'!$A$1:$D$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Modules'!$A$1:$C$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Modules'!$A$1:$C$110</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Roadmap'!$A$1:$F$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5">
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11">
@@ -548,7 +548,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>29710</v>
+        <v>30150</v>
       </c>
     </row>
     <row r="12">
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -617,7 +617,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="20">
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
@@ -740,21 +740,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>metadata</t>
+          <t>runtime</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>runtime</t>
+          <t>metadata</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="35">
@@ -1379,20 +1379,24 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>not built</t>
+          <t>partial</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>No spatial chunking exists. The agent layer batches features by vertex weight to keep memory bounded; that is a batching strategy, not a spatial tiling, and it does not preserve topology across batches.</t>
+          <t>Halo-buffered tiling in geoqa/chunking.py. A tile selects every feature intersecting its bounds plus a declared halo, geometries whole and never clipped, so a feature crossing a boundary is validated identically on both sides. Findings are deduplicated on problem name and feature id.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>A tiled implementation must buffer each tile by a halo so a feature crossing a boundary is present on both sides, otherwise connectivity checks report false breaks at the seams. Whole-layer union and degree checks cannot be tiled at all and need a single global pass. Until both exist, any large-layer run must complete in one pass.</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
+          <t>An undeclared halo on a multi-tile run is reported as evidence rather than passing silently. scripts/verify_chunking_equivalence.py demonstrates the property: with a halo, a 64-tile run returns exactly the findings the whole-layer run returns; with the halo removed the same run invents one. Not yet wired into validation_runtime dispatch, and the budget is a vertex count rather than a measured memory ceiling.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Chunking is opt-in per validator: a validator runs on the whole layer unless it is named in CHUNK_LOCAL_VALIDATORS, because whole-layer correctness is the default and tiling has to earn the right to change what a validator can see. Twelve validators are declared tileable; the topology questions cannot be tiled at all and are listed with the reason.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1613,7 +1617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J254"/>
+  <dimension ref="A1:J256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10412,17 +10416,17 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>hardware_cpu_throttled</t>
+          <t>chunk_halo_undeclared</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>runtime_issue</t>
+          <t>evidence_condition</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
@@ -10438,12 +10442,12 @@
       <c r="G183" t="inlineStr"/>
       <c r="H183" t="inlineStr">
         <is>
-          <t>The processor is running materially below its rated clock, so a runtime measured elsewhere does not apply and an apparent timeout is more likely to be this than a bug.</t>
+          <t>A multi-tile validation run was performed with no halo, so features either side of a tile boundary were never validated together and topology findings on that run cannot be trusted.</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>Cool down, reduce parallelism, or allow more time. Do not treat the slowdown as a code defect before ruling this out.</t>
+          <t>Declare a halo at least as wide as the largest feature-to-feature distance the caller is prepared to call a break, or run the affected validators on the whole layer. Do not read topology findings from an unhaloed run.</t>
         </is>
       </c>
       <c r="J183" t="inlineStr"/>
@@ -10456,17 +10460,17 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>hardware_disk_space_insufficient</t>
+          <t>chunk_validator_not_tileable</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>info</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>runtime_issue</t>
+          <t>evidence_condition</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
@@ -10476,18 +10480,18 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G184" t="inlineStr"/>
       <c r="H184" t="inlineStr">
         <is>
-          <t>The write would leave the volume below the declared free fraction. Filling a volume tends to break other software on the machine at the same time, not just this run.</t>
+          <t>A validator was run on the whole layer because the question it asks cannot be answered from a tile.</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>Free space, write to another volume, or extract selectively rather than unpacking everything.</t>
+          <t>No action is needed if the whole-layer run is intended. If the caller expected this validator to be tiled, the expectation is wrong rather than the code.</t>
         </is>
       </c>
       <c r="J184" t="inlineStr"/>
@@ -10500,12 +10504,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>hardware_memory_insufficient</t>
+          <t>hardware_cpu_throttled</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -10526,12 +10530,12 @@
       <c r="G185" t="inlineStr"/>
       <c r="H185" t="inlineStr">
         <is>
-          <t>The operation needs more memory than is available, leaving less than the declared headroom. This fails partway through rather than at the start, which is the worst time.</t>
+          <t>The processor is running materially below its rated clock, so a runtime measured elsewhere does not apply and an apparent timeout is more likely to be this than a bug.</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>Read the data in windows, reduce the resolution, or defer the operation. Windowed reads exist for exactly this case.</t>
+          <t>Cool down, reduce parallelism, or allow more time. Do not treat the slowdown as a code defect before ruling this out.</t>
         </is>
       </c>
       <c r="J185" t="inlineStr"/>
@@ -10544,12 +10548,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>hardware_temperature_unavailable</t>
+          <t>hardware_disk_space_insufficient</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -10570,12 +10574,12 @@
       <c r="G186" t="inlineStr"/>
       <c r="H186" t="inlineStr">
         <is>
-          <t>No core temperature could be read, so no thermal limit can be enforced for this run.</t>
+          <t>The write would leave the volume below the declared free fraction. Filling a volume tends to break other software on the machine at the same time, not just this run.</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>On Windows, install LibreHardwareMonitor and run it once so its WMI namespace exists. On Linux, /sys/class/hwmon is the native interface and needs nothing installed; install lm-sensors only if the kernel exposes no CPU chip.</t>
+          <t>Free space, write to another volume, or extract selectively rather than unpacking everything.</t>
         </is>
       </c>
       <c r="J186" t="inlineStr"/>
@@ -10588,12 +10592,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>raster_block_size_small</t>
+          <t>hardware_memory_insufficient</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -10603,23 +10607,23 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G187" t="inlineStr"/>
       <c r="H187" t="inlineStr">
         <is>
-          <t>Tiles are smaller than the 512 px convention, increasing metadata overhead without improving access, since a partial read still costs a whole tile.</t>
+          <t>The operation needs more memory than is available, leaving less than the declared headroom. This fails partway through rather than at the start, which is the worst time.</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>Use 512 px tiles unless a specific workload justifies otherwise.</t>
+          <t>Read the data in windows, reduce the resolution, or defer the operation. Windowed reads exist for exactly this case.</t>
         </is>
       </c>
       <c r="J187" t="inlineStr"/>
@@ -10632,12 +10636,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>raster_missing_overviews</t>
+          <t>hardware_temperature_unavailable</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -10658,12 +10662,12 @@
       <c r="G188" t="inlineStr"/>
       <c r="H188" t="inlineStr">
         <is>
-          <t>A large TIFF has no reduced-resolution overview levels, so a consumer must read full resolution to draw a thumbnail.</t>
+          <t>No core temperature could be read, so no thermal limit can be enforced for this run.</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>Build overviews when writing. This is the main reason cloud-optimized layouts exist.</t>
+          <t>On Windows, install LibreHardwareMonitor and run it once so its WMI namespace exists. On Linux, /sys/class/hwmon is the native interface and needs nothing installed; install lm-sensors only if the kernel exposes no CPU chip.</t>
         </is>
       </c>
       <c r="J188" t="inlineStr"/>
@@ -10676,38 +10680,38 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>raster_not_cloud_optimized</t>
+          <t>raster_block_size_small</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>runtime_issue</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="D189" t="inlineStr">
-        <is>
-          <t>runtime_issue</t>
-        </is>
-      </c>
-      <c r="E189" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G189" t="inlineStr"/>
       <c r="H189" t="inlineStr">
         <is>
-          <t>A large TIFF is stored in strips rather than tiles. It is valid and opens everywhere, but a reader cannot fetch a small part of it, so anything serving it over a network must move the whole file.</t>
+          <t>Tiles are smaller than the 512 px convention, increasing metadata overhead without improving access, since a partial read still costs a whole tile.</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>Rewrite as a Cloud Optimized GeoTIFF. Legacy readers still open a COG, so there is no compatibility cost.</t>
+          <t>Use 512 px tiles unless a specific workload justifies otherwise.</t>
         </is>
       </c>
       <c r="J189" t="inlineStr"/>
@@ -10720,7 +10724,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>runtime_limit_exceeded</t>
+          <t>raster_missing_overviews</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -10746,12 +10750,12 @@
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr">
         <is>
-          <t>Validation stopped early because the configured runtime ceiling was reached.</t>
+          <t>A large TIFF has no reduced-resolution overview levels, so a consumer must read full resolution to draw a thumbnail.</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>Rerun with a larger runtime budget, narrower profile, or smaller/adaptive chunks.</t>
+          <t>Build overviews when writing. This is the main reason cloud-optimized layouts exist.</t>
         </is>
       </c>
       <c r="J190" t="inlineStr"/>
@@ -10764,7 +10768,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>workbook_media_undecodable</t>
+          <t>raster_not_cloud_optimized</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -10774,7 +10778,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>evidence_condition</t>
+          <t>runtime_issue</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -10790,12 +10794,12 @@
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="inlineStr">
         <is>
-          <t>An attachment is in a format that cannot be inspected here, so it is unverified rather than checked.</t>
+          <t>A large TIFF is stored in strips rather than tiles. It is valid and opens everywhere, but a reader cannot fetch a small part of it, so anything serving it over a network must move the whole file.</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>Convert to a format that can be validated, or verify it by another means and record that it was verified.</t>
+          <t>Rewrite as a Cloud Optimized GeoTIFF. Legacy readers still open a COG, so there is no compatibility cost.</t>
         </is>
       </c>
       <c r="J191" t="inlineStr"/>
@@ -10808,17 +10812,17 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>workbook_no_attachments</t>
+          <t>runtime_limit_exceeded</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>evidence_condition</t>
+          <t>runtime_issue</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -10828,18 +10832,18 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G192" t="inlineStr"/>
       <c r="H192" t="inlineStr">
         <is>
-          <t>The workbook holds no attachments at all.</t>
+          <t>Validation stopped early because the configured runtime ceiling was reached.</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>Establish this before concluding that supporting evidence is missing.</t>
+          <t>Rerun with a larger runtime budget, narrower profile, or smaller/adaptive chunks.</t>
         </is>
       </c>
       <c r="J192" t="inlineStr"/>
@@ -10847,12 +10851,12 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>schema</t>
+          <t>runtime</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>coordinate_axis_order_non_numeric</t>
+          <t>workbook_media_undecodable</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -10862,7 +10866,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>schema_defect</t>
+          <t>evidence_condition</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
@@ -10878,12 +10882,12 @@
       <c r="G193" t="inlineStr"/>
       <c r="H193" t="inlineStr">
         <is>
-          <t>A coordinate column holds values that are not numbers. These rows cannot be checked and will disappear silently on upload.</t>
+          <t>An attachment is in a format that cannot be inspected here, so it is unverified rather than checked.</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>Correct the values at source and re-ingest. Text in a numeric column is usually an error code or a stray delimiter.</t>
+          <t>Convert to a format that can be validated, or verify it by another means and record that it was verified.</t>
         </is>
       </c>
       <c r="J193" t="inlineStr"/>
@@ -10891,22 +10895,22 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>schema</t>
+          <t>runtime</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>epanet_non_numeric_field</t>
+          <t>workbook_no_attachments</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>info</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>schema_defect</t>
+          <t>evidence_condition</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
@@ -10916,18 +10920,18 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G194" t="inlineStr"/>
       <c r="H194" t="inlineStr">
         <is>
-          <t>A field that EPANET parses as a number contains a non-numeric value.</t>
+          <t>The workbook holds no attachments at all.</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>Correct the value or quote the field if EPANET treats it as a comment for this section.</t>
+          <t>Establish this before concluding that supporting evidence is missing.</t>
         </is>
       </c>
       <c r="J194" t="inlineStr"/>
@@ -10940,7 +10944,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>json_in_text_column</t>
+          <t>coordinate_axis_order_non_numeric</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -10966,12 +10970,12 @@
       <c r="G195" t="inlineStr"/>
       <c r="H195" t="inlineStr">
         <is>
-          <t>A column declared as text contains a serialised JSON structure. Unstructured data in a typed field defeats type checking, validation and aggregation.</t>
+          <t>A coordinate column holds values that are not numbers. These rows cannot be checked and will disappear silently on upload.</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>Parse the payload into typed columns, or keep it as text and validate that it parses on every row. Consumers currently rely on hand-written tolerant parsers.</t>
+          <t>Correct the values at source and re-ingest. Text in a numeric column is usually an error code or a stray delimiter.</t>
         </is>
       </c>
       <c r="J195" t="inlineStr"/>
@@ -10984,7 +10988,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>json_in_text_unparseable</t>
+          <t>epanet_non_numeric_field</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -11010,12 +11014,12 @@
       <c r="G196" t="inlineStr"/>
       <c r="H196" t="inlineStr">
         <is>
-          <t>A column contains what looks like a JSON payload but at least one row fails to parse, so the vendor format has changed or the row is corrupt.</t>
+          <t>A field that EPANET parses as a number contains a non-numeric value.</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>Identify the row that breaks the parse. Treat downstream readers of this column as unreliable until it is fixed.</t>
+          <t>Correct the value or quote the field if EPANET treats it as a comment for this section.</t>
         </is>
       </c>
       <c r="J196" t="inlineStr"/>
@@ -11028,7 +11032,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>tabular_blank_header</t>
+          <t>json_in_text_column</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -11054,12 +11058,12 @@
       <c r="G197" t="inlineStr"/>
       <c r="H197" t="inlineStr">
         <is>
-          <t>A column has no name and will be imported as an unnamed column, so its values have nothing to be referred to by.</t>
+          <t>A column declared as text contains a serialised JSON structure. Unstructured data in a typed field defeats type checking, validation and aggregation.</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>Name the column. Where the values were never meant to be data, remove the column.</t>
+          <t>Parse the payload into typed columns, or keep it as text and validate that it parses on every row. Consumers currently rely on hand-written tolerant parsers.</t>
         </is>
       </c>
       <c r="J197" t="inlineStr"/>
@@ -11072,7 +11076,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>tabular_duplicate_header</t>
+          <t>json_in_text_unparseable</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -11098,12 +11102,12 @@
       <c r="G198" t="inlineStr"/>
       <c r="H198" t="inlineStr">
         <is>
-          <t>Two or more columns share a name, so a lookup by that name returns an arbitrary one of them.</t>
+          <t>A column contains what looks like a JSON payload but at least one row fails to parse, so the vendor format has changed or the row is corrupt.</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>Rename to unique names before any automated processing.</t>
+          <t>Identify the row that breaks the parse. Treat downstream readers of this column as unreliable until it is fixed.</t>
         </is>
       </c>
       <c r="J198" t="inlineStr"/>
@@ -11116,12 +11120,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>tabular_empty_column</t>
+          <t>tabular_blank_header</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -11142,12 +11146,12 @@
       <c r="G199" t="inlineStr"/>
       <c r="H199" t="inlineStr">
         <is>
-          <t>A column is empty in every row.</t>
+          <t>A column has no name and will be imported as an unnamed column, so its values have nothing to be referred to by.</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>Remove the column, or populate it. Either way, confirm it was not meant to carry data.</t>
+          <t>Name the column. Where the values were never meant to be data, remove the column.</t>
         </is>
       </c>
       <c r="J199" t="inlineStr"/>
@@ -11160,12 +11164,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>tabular_formula_cells</t>
+          <t>tabular_duplicate_header</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -11186,12 +11190,12 @@
       <c r="G200" t="inlineStr"/>
       <c r="H200" t="inlineStr">
         <is>
-          <t>Cells hold formulas. A reader that does not evaluate them sees the last cached value, which may be out of date.</t>
+          <t>Two or more columns share a name, so a lookup by that name returns an arbitrary one of them.</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>Paste as values before processing, or read the cached results knowingly as potentially stale.</t>
+          <t>Rename to unique names before any automated processing.</t>
         </is>
       </c>
       <c r="J200" t="inlineStr"/>
@@ -11204,12 +11208,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>tabular_hidden_rows</t>
+          <t>tabular_empty_column</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -11230,12 +11234,12 @@
       <c r="G201" t="inlineStr"/>
       <c r="H201" t="inlineStr">
         <is>
-          <t>Rows are hidden and will not appear in a default read.</t>
+          <t>A column is empty in every row.</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Confirm whether the hidden rows are excluded deliberately or were hidden to hide an error.</t>
+          <t>Remove the column, or populate it. Either way, confirm it was not meant to carry data.</t>
         </is>
       </c>
       <c r="J201" t="inlineStr"/>
@@ -11248,12 +11252,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>tabular_hidden_sheet</t>
+          <t>tabular_formula_cells</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -11274,12 +11278,12 @@
       <c r="G202" t="inlineStr"/>
       <c r="H202" t="inlineStr">
         <is>
-          <t>A sheet is hidden and will not appear in a default read, so whatever corrections it holds look as though they were never made.</t>
+          <t>Cells hold formulas. A reader that does not evaluate them sees the last cached value, which may be out of date.</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>Read every sheet explicitly, or unhide the sheets that carry data.</t>
+          <t>Paste as values before processing, or read the cached results knowingly as potentially stale.</t>
         </is>
       </c>
       <c r="J202" t="inlineStr"/>
@@ -11292,12 +11296,12 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>tabular_identifier_leading_zero</t>
+          <t>tabular_hidden_rows</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -11318,12 +11322,12 @@
       <c r="G203" t="inlineStr"/>
       <c r="H203" t="inlineStr">
         <is>
-          <t>An identifier-like column holds all-numeric values with a leading zero. Reading it as a number destroys the identifier and the records will never match the source system.</t>
+          <t>Rows are hidden and will not appear in a default read.</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>Force the column to text at export and at every read. A repair that re-pads the number cannot know whether the original had the zero.</t>
+          <t>Confirm whether the hidden rows are excluded deliberately or were hidden to hide an error.</t>
         </is>
       </c>
       <c r="J203" t="inlineStr"/>
@@ -11336,7 +11340,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>tabular_identifier_numeric</t>
+          <t>tabular_hidden_sheet</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -11362,12 +11366,12 @@
       <c r="G204" t="inlineStr"/>
       <c r="H204" t="inlineStr">
         <is>
-          <t>An identifier is held as a number with enough digits that spreadsheet software renders it in scientific notation and rounds the low digits.</t>
+          <t>A sheet is hidden and will not appear in a default read, so whatever corrections it holds look as though they were never made.</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>Store identifiers as text. Precision loss in an identifier is silent and permanent.</t>
+          <t>Read every sheet explicitly, or unhide the sheets that carry data.</t>
         </is>
       </c>
       <c r="J204" t="inlineStr"/>
@@ -11380,12 +11384,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>tabular_merged_cells</t>
+          <t>tabular_identifier_leading_zero</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -11406,12 +11410,12 @@
       <c r="G205" t="inlineStr"/>
       <c r="H205" t="inlineStr">
         <is>
-          <t>Merged cells store their value only on the top-left cell, so every other row reads as empty and any group-by or filter over that column drops them.</t>
+          <t>An identifier-like column holds all-numeric values with a leading zero. Reading it as a number destroys the identifier and the records will never match the source system.</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Unmerge and repeat the value on each row before any automated processing.</t>
+          <t>Force the column to text at export and at every read. A repair that re-pads the number cannot know whether the original had the zero.</t>
         </is>
       </c>
       <c r="J205" t="inlineStr"/>
@@ -11424,7 +11428,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>tabular_missing_expected_column</t>
+          <t>tabular_identifier_numeric</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -11450,12 +11454,12 @@
       <c r="G206" t="inlineStr"/>
       <c r="H206" t="inlineStr">
         <is>
-          <t>A column the caller expected is absent from the file.</t>
+          <t>An identifier is held as a number with enough digits that spreadsheet software renders it in scientific notation and rounds the low digits.</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Check the export configuration. A renamed column changes every reference to it.</t>
+          <t>Store identifiers as text. Precision loss in an identifier is silent and permanent.</t>
         </is>
       </c>
       <c r="J206" t="inlineStr"/>
@@ -11468,7 +11472,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>tabular_missing_header</t>
+          <t>tabular_merged_cells</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -11494,12 +11498,12 @@
       <c r="G207" t="inlineStr"/>
       <c r="H207" t="inlineStr">
         <is>
-          <t>The file has no readable header row, so columns will be named positionally and every downstream reference to a column name fails.</t>
+          <t>Merged cells store their value only on the top-left cell, so every other row reads as empty and any group-by or filter over that column drops them.</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Add a header row and re-export. Positional column names cannot be joined against anything.</t>
+          <t>Unmerge and repeat the value on each row before any automated processing.</t>
         </is>
       </c>
       <c r="J207" t="inlineStr"/>
@@ -11512,7 +11516,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>tabular_ragged_rows</t>
+          <t>tabular_missing_expected_column</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -11538,12 +11542,12 @@
       <c r="G208" t="inlineStr"/>
       <c r="H208" t="inlineStr">
         <is>
-          <t>Some rows have a different column count from the header. The surplus or missing values shift into neighbouring columns without raising an error.</t>
+          <t>A column the caller expected is absent from the file.</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Re-export with a consistent column count, and find the source of the unescaped delimiter before doing so.</t>
+          <t>Check the export configuration. A renamed column changes every reference to it.</t>
         </is>
       </c>
       <c r="J208" t="inlineStr"/>
@@ -11556,22 +11560,22 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>workbook_media_duplicate</t>
+          <t>tabular_missing_header</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>data_issue</t>
+          <t>schema_defect</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
@@ -11582,12 +11586,12 @@
       <c r="G209" t="inlineStr"/>
       <c r="H209" t="inlineStr">
         <is>
-          <t>Identical attachment content appears more than once, usually a copy-paste artefact, and usually two records pointing at one piece of evidence.</t>
+          <t>The file has no readable header row, so columns will be named positionally and every downstream reference to a column name fails.</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>Confirm each record has its own evidence. Two rows sharing one attachment is a finding about the data, not about the file.</t>
+          <t>Add a header row and re-export. Positional column names cannot be joined against anything.</t>
         </is>
       </c>
       <c r="J209" t="inlineStr"/>
@@ -11600,12 +11604,12 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>workbook_media_orphaned</t>
+          <t>tabular_ragged_rows</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -11626,12 +11630,12 @@
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="inlineStr">
         <is>
-          <t>An attachment is embedded but anchored to no row, so it documents nothing.</t>
+          <t>Some rows have a different column count from the header. The surplus or missing values shift into neighbouring columns without raising an error.</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>Anchor the attachment to the row it belongs to, or remove it.</t>
+          <t>Re-export with a consistent column count, and find the source of the unescaped delimiter before doing so.</t>
         </is>
       </c>
       <c r="J210" t="inlineStr"/>
@@ -11644,22 +11648,22 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>workbook_media_unverifiable</t>
+          <t>workbook_media_duplicate</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>schema_defect</t>
+          <t>data_issue</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
@@ -11670,12 +11674,12 @@
       <c r="G211" t="inlineStr"/>
       <c r="H211" t="inlineStr">
         <is>
-          <t>The key column is absent, so no attachment can be traced back to a record.</t>
+          <t>Identical attachment content appears more than once, usually a copy-paste artefact, and usually two records pointing at one piece of evidence.</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>Supply or restore the identifier column.</t>
+          <t>Confirm each record has its own evidence. Two rows sharing one attachment is a finding about the data, not about the file.</t>
         </is>
       </c>
       <c r="J211" t="inlineStr"/>
@@ -11683,22 +11687,22 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>spatial_logic</t>
+          <t>schema</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>clip_straddles_boundary</t>
+          <t>workbook_media_orphaned</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>evidence_condition</t>
+          <t>schema_defect</t>
         </is>
       </c>
       <c r="E212" t="inlineStr">
@@ -11708,18 +11712,18 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr">
         <is>
-          <t>A feature crosses a boundary, with a measured split between the two sides. Evidence, not a defect: the point is that the decision is visible.</t>
+          <t>An attachment is embedded but anchored to no row, so it documents nothing.</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>Confirm the assigned side is the intended one under the declared threshold.</t>
+          <t>Anchor the attachment to the row it belongs to, or remove it.</t>
         </is>
       </c>
       <c r="J212" t="inlineStr"/>
@@ -11727,12 +11731,12 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>spatial_logic</t>
+          <t>schema</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>line_intersection_other_layer</t>
+          <t>workbook_media_unverifiable</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -11742,12 +11746,12 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>data_issue</t>
+          <t>schema_defect</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
@@ -11758,19 +11762,15 @@
       <c r="G213" t="inlineStr"/>
       <c r="H213" t="inlineStr">
         <is>
-          <t>Lines intersect features in another layer where crossing is not permitted by the data model.</t>
+          <t>The key column is absent, so no attachment can be traced back to a record.</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>Review the crossing rule and either create a valid junction or reroute the feature to avoid the prohibited crossing.</t>
-        </is>
-      </c>
-      <c r="J213" t="inlineStr">
-        <is>
-          <t>QGIS Topology Checker Plugin</t>
-        </is>
-      </c>
+          <t>Supply or restore the identifier column.</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -11780,45 +11780,41 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>point_not_coincident_with_point</t>
+          <t>clip_straddles_boundary</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>info</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>data_issue</t>
+          <t>evidence_condition</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G214" t="inlineStr"/>
       <c r="H214" t="inlineStr">
         <is>
-          <t>A point feature should align with a corresponding point in another layer but does not.</t>
+          <t>A feature crosses a boundary, with a measured split between the two sides. Evidence, not a defect: the point is that the decision is visible.</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>Snap the point to the authoritative location or adjust the paired feature so both coincide.</t>
-        </is>
-      </c>
-      <c r="J214" t="inlineStr">
-        <is>
-          <t>ArcGIS Geodatabase Topology Rules</t>
-        </is>
-      </c>
+          <t>Confirm the assigned side is the intended one under the declared threshold.</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -11828,7 +11824,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>point_not_covered_by_line</t>
+          <t>line_intersection_other_layer</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -11854,12 +11850,12 @@
       <c r="G215" t="inlineStr"/>
       <c r="H215" t="inlineStr">
         <is>
-          <t>A point that should coincide with a line is not located on any line feature.</t>
+          <t>Lines intersect features in another layer where crossing is not permitted by the data model.</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>Snap the point to the correct line or correct the point placement using a reference layer.</t>
+          <t>Review the crossing rule and either create a valid junction or reroute the feature to avoid the prohibited crossing.</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
@@ -11876,7 +11872,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>point_not_inside_polygon</t>
+          <t>point_not_coincident_with_point</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -11902,17 +11898,17 @@
       <c r="G216" t="inlineStr"/>
       <c r="H216" t="inlineStr">
         <is>
-          <t>A point expected to fall inside a polygon lies outside the target area.</t>
+          <t>A point feature should align with a corresponding point in another layer but does not.</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>Move the point into the correct polygon or repair the polygon boundary if the point placement is already trusted.</t>
+          <t>Snap the point to the authoritative location or adjust the paired feature so both coincide.</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
         <is>
-          <t>QGIS Topology Checker Plugin</t>
+          <t>ArcGIS Geodatabase Topology Rules</t>
         </is>
       </c>
     </row>
@@ -11924,7 +11920,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>polygon_boundary_mismatch</t>
+          <t>point_not_covered_by_line</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -11950,12 +11946,12 @@
       <c r="G217" t="inlineStr"/>
       <c r="H217" t="inlineStr">
         <is>
-          <t>A polygon boundary is not fully covered by the matching linework or other polygon boundaries.</t>
+          <t>A point that should coincide with a line is not located on any line feature.</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>Use snapping or shared-boundary editing so polygon boundaries align exactly with the reference linework.</t>
+          <t>Snap the point to the correct line or correct the point placement using a reference layer.</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
@@ -11972,7 +11968,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>polygon_boundary_not_covered_by_lines</t>
+          <t>point_not_inside_polygon</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -11998,17 +11994,17 @@
       <c r="G218" t="inlineStr"/>
       <c r="H218" t="inlineStr">
         <is>
-          <t>Polygon boundaries should match a line layer but some boundary segments have no corresponding line.</t>
+          <t>A point expected to fall inside a polygon lies outside the target area.</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>Generate or edit missing boundary lines so the polygon perimeter is fully represented.</t>
+          <t>Move the point into the correct polygon or repair the polygon boundary if the point placement is already trusted.</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
         <is>
-          <t>ArcGIS Geodatabase Topology Rules</t>
+          <t>QGIS Topology Checker Plugin</t>
         </is>
       </c>
     </row>
@@ -12020,7 +12016,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>polygon_missing_contained_point</t>
+          <t>polygon_boundary_mismatch</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -12046,17 +12042,17 @@
       <c r="G219" t="inlineStr"/>
       <c r="H219" t="inlineStr">
         <is>
-          <t>A polygon expected to contain at least one related point contains none.</t>
+          <t>A polygon boundary is not fully covered by the matching linework or other polygon boundaries.</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>Create the missing point or move an existing related point into the polygon if one should already exist.</t>
+          <t>Use snapping or shared-boundary editing so polygon boundaries align exactly with the reference linework.</t>
         </is>
       </c>
       <c r="J219" t="inlineStr">
         <is>
-          <t>ArcGIS Geodatabase Topology Rules</t>
+          <t>QGIS Topology Checker Plugin</t>
         </is>
       </c>
     </row>
@@ -12068,7 +12064,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>polygon_not_covered_by_other_polygons</t>
+          <t>polygon_boundary_not_covered_by_lines</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -12094,12 +12090,12 @@
       <c r="G220" t="inlineStr"/>
       <c r="H220" t="inlineStr">
         <is>
-          <t>A polygon should be fully covered by another polygon class, but parts of it fall outside coverage.</t>
+          <t>Polygon boundaries should match a line layer but some boundary segments have no corresponding line.</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>Expand or correct the covering layer so the target polygon is fully covered where business rules require it.</t>
+          <t>Generate or edit missing boundary lines so the polygon perimeter is fully represented.</t>
         </is>
       </c>
       <c r="J220" t="inlineStr">
@@ -12116,7 +12112,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>polygon_overlap_other_layer</t>
+          <t>polygon_missing_contained_point</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -12142,12 +12138,12 @@
       <c r="G221" t="inlineStr"/>
       <c r="H221" t="inlineStr">
         <is>
-          <t>Polygons from different classes overlap even though the same space should not belong to both classes.</t>
+          <t>A polygon expected to contain at least one related point contains none.</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>Review class rules and edit one or both layers so only the correct polygon retains the overlapping area.</t>
+          <t>Create the missing point or move an existing related point into the polygon if one should already exist.</t>
         </is>
       </c>
       <c r="J221" t="inlineStr">
@@ -12164,7 +12160,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>polygon_point_count_mismatch</t>
+          <t>polygon_not_covered_by_other_polygons</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -12190,12 +12186,12 @@
       <c r="G222" t="inlineStr"/>
       <c r="H222" t="inlineStr">
         <is>
-          <t>The polygon-to-point relationship violates a required one-to-one correspondence.</t>
+          <t>A polygon should be fully covered by another polygon class, but parts of it fall outside coverage.</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>Audit related point records and add, remove, or reassign points until the required count rule is satisfied.</t>
+          <t>Expand or correct the covering layer so the target polygon is fully covered where business rules require it.</t>
         </is>
       </c>
       <c r="J222" t="inlineStr">
@@ -12212,7 +12208,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>polygons_do_not_cover_each_other</t>
+          <t>polygon_overlap_other_layer</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -12238,12 +12234,12 @@
       <c r="G223" t="inlineStr"/>
       <c r="H223" t="inlineStr">
         <is>
-          <t>Two polygon classifications intended to represent the same space do not fully correspond.</t>
+          <t>Polygons from different classes overlap even though the same space should not belong to both classes.</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>Compare both polygon coverages and repair gaps or mismatches through snapping, union, or shared-boundary editing.</t>
+          <t>Review class rules and edit one or both layers so only the correct polygon retains the overlapping area.</t>
         </is>
       </c>
       <c r="J223" t="inlineStr">
@@ -12260,12 +12256,12 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>unsnapped_vertices_within_tolerance</t>
+          <t>polygon_point_count_mismatch</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -12286,29 +12282,29 @@
       <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr">
         <is>
-          <t>Vertices that should align to a reference geometry remain slightly offset within an expected snapping tolerance. Diagnose by running snapping tools against the reference layer and review whether new vertices must be inserted.</t>
+          <t>The polygon-to-point relationship violates a required one-to-one correspondence.</t>
         </is>
       </c>
       <c r="I224" t="inlineStr">
         <is>
-          <t>Run snapping tools against the reference layer using an appropriate tolerance.</t>
+          <t>Audit related point records and add, remove, or reassign points until the required count rule is satisfied.</t>
         </is>
       </c>
       <c r="J224" t="inlineStr">
         <is>
-          <t>QGIS Vector Geometry Algorithms</t>
+          <t>ArcGIS Geodatabase Topology Rules</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>topology</t>
+          <t>spatial_logic</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>continuity_break</t>
+          <t>polygons_do_not_cover_each_other</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -12331,37 +12327,37 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G225" t="inlineStr">
-        <is>
-          <t>Logical Consistency</t>
-        </is>
-      </c>
+      <c r="G225" t="inlineStr"/>
       <c r="H225" t="inlineStr">
         <is>
-          <t>A line referenced as continuous is broken into disconnected parts within its own declared tolerance.</t>
+          <t>Two polygon classifications intended to represent the same space do not fully correspond.</t>
         </is>
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>Confirm whether the break is a real gap or a digitising artefact, then either repair the line or restate the declared tolerance.</t>
-        </is>
-      </c>
-      <c r="J225" t="inlineStr"/>
+          <t>Compare both polygon coverages and repair gaps or mismatches through snapping, union, or shared-boundary editing.</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>ArcGIS Geodatabase Topology Rules</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>topology</t>
+          <t>spatial_logic</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>dma_cross_name_equal_geometry</t>
+          <t>unsnapped_vertices_within_tolerance</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -12371,7 +12367,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
@@ -12379,22 +12375,22 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G226" t="inlineStr">
-        <is>
-          <t>Logical Consistency</t>
-        </is>
-      </c>
+      <c r="G226" t="inlineStr"/>
       <c r="H226" t="inlineStr">
         <is>
-          <t>Two different DMA names map to effectively the same polygon geometry.</t>
+          <t>Vertices that should align to a reference geometry remain slightly offset within an expected snapping tolerance. Diagnose by running snapping tools against the reference layer and review whether new vertices must be inserted.</t>
         </is>
       </c>
       <c r="I226" t="inlineStr">
         <is>
-          <t>Resolve the naming conflict before deciding which geometry or label should be retained.</t>
-        </is>
-      </c>
-      <c r="J226" t="inlineStr"/>
+          <t>Run snapping tools against the reference layer using an appropriate tolerance.</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>QGIS Vector Geometry Algorithms</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -12404,7 +12400,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>dma_cross_name_nested_polygon</t>
+          <t>continuity_break</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -12419,7 +12415,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
@@ -12434,12 +12430,12 @@
       </c>
       <c r="H227" t="inlineStr">
         <is>
-          <t>A DMA polygon is nearly fully nested inside a differently named DMA polygon.</t>
+          <t>A line referenced as continuous is broken into disconnected parts within its own declared tolerance.</t>
         </is>
       </c>
       <c r="I227" t="inlineStr">
         <is>
-          <t>Inspect the naming conflict and nested coverage before merging, subtracting, or retiring one polygon.</t>
+          <t>Confirm whether the break is a real gap or a digitising artefact, then either repair the line or restate the declared tolerance.</t>
         </is>
       </c>
       <c r="J227" t="inlineStr"/>
@@ -12452,7 +12448,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>dma_cross_name_overlap</t>
+          <t>dma_cross_name_equal_geometry</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -12482,12 +12478,12 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>Two differently named DMA polygons partially overlap.</t>
+          <t>Two different DMA names map to effectively the same polygon geometry.</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
         <is>
-          <t>Review which polygon should own the overlap and resolve it using subtraction or a controlled merge.</t>
+          <t>Resolve the naming conflict before deciding which geometry or label should be retained.</t>
         </is>
       </c>
       <c r="J228" t="inlineStr"/>
@@ -12500,12 +12496,12 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>dma_multipart_polygon</t>
+          <t>dma_cross_name_nested_polygon</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -12515,7 +12511,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
@@ -12530,12 +12526,12 @@
       </c>
       <c r="H229" t="inlineStr">
         <is>
-          <t>A DMA is split across multiple polygon parts after explode(), indicating fragmentation or multipart coverage.</t>
+          <t>A DMA polygon is nearly fully nested inside a differently named DMA polygon.</t>
         </is>
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>Inspect whether the same-name polygon fragments should be dissolved into a single retained feature.</t>
+          <t>Inspect the naming conflict and nested coverage before merging, subtracting, or retiring one polygon.</t>
         </is>
       </c>
       <c r="J229" t="inlineStr"/>
@@ -12548,7 +12544,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>dma_same_name_equal_geometry</t>
+          <t>dma_cross_name_overlap</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -12578,12 +12574,12 @@
       </c>
       <c r="H230" t="inlineStr">
         <is>
-          <t>Two same-name DMA polygons are geometrically equal and likely duplicate one another.</t>
+          <t>Two differently named DMA polygons partially overlap.</t>
         </is>
       </c>
       <c r="I230" t="inlineStr">
         <is>
-          <t>Inspect the duplicate same-name polygons and dissolve or retire the redundant feature if the duplication is unintended.</t>
+          <t>Review which polygon should own the overlap and resolve it using subtraction or a controlled merge.</t>
         </is>
       </c>
       <c r="J230" t="inlineStr"/>
@@ -12596,12 +12592,12 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>dma_same_name_nested_polygon</t>
+          <t>dma_multipart_polygon</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -12611,7 +12607,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
@@ -12626,12 +12622,12 @@
       </c>
       <c r="H231" t="inlineStr">
         <is>
-          <t>Two same-name DMA polygons are almost fully nested, indicating duplicate or fragmented coverage.</t>
+          <t>A DMA is split across multiple polygon parts after explode(), indicating fragmentation or multipart coverage.</t>
         </is>
       </c>
       <c r="I231" t="inlineStr">
         <is>
-          <t>Review the nested same-name polygons and dissolve or remove the smaller duplicate if appropriate.</t>
+          <t>Inspect whether the same-name polygon fragments should be dissolved into a single retained feature.</t>
         </is>
       </c>
       <c r="J231" t="inlineStr"/>
@@ -12644,7 +12640,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>duplicate_feature_geometry</t>
+          <t>dma_same_name_equal_geometry</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -12674,19 +12670,15 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>Two or more features have the same geometry, creating duplicate spatial records.</t>
+          <t>Two same-name DMA polygons are geometrically equal and likely duplicate one another.</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
         <is>
-          <t>Find duplicate shapes and keep the authoritative record while deleting or merging duplicates.</t>
-        </is>
-      </c>
-      <c r="J232" t="inlineStr">
-        <is>
-          <t>QGIS Geometry Checker Plugin</t>
-        </is>
-      </c>
+          <t>Inspect the duplicate same-name polygons and dissolve or retire the redundant feature if the duplication is unintended.</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -12696,12 +12688,12 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>duplicate_geometry_same_layer</t>
+          <t>dma_same_name_nested_polygon</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -12726,12 +12718,12 @@
       </c>
       <c r="H233" t="inlineStr">
         <is>
-          <t>A feature duplicates the geometry of another feature in the same layer.</t>
+          <t>Two same-name DMA polygons are almost fully nested, indicating duplicate or fragmented coverage.</t>
         </is>
       </c>
       <c r="I233" t="inlineStr">
         <is>
-          <t>Review whether duplicate features should be merged, deleted, or linked by shared identifiers.</t>
+          <t>Review the nested same-name polygons and dissolve or remove the smaller duplicate if appropriate.</t>
         </is>
       </c>
       <c r="J233" t="inlineStr"/>
@@ -12744,7 +12736,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>duplicate_point</t>
+          <t>duplicate_feature_geometry</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -12774,17 +12766,17 @@
       </c>
       <c r="H234" t="inlineStr">
         <is>
-          <t>Multiple points occupy the same location where duplicates are not allowed.</t>
+          <t>Two or more features have the same geometry, creating duplicate spatial records.</t>
         </is>
       </c>
       <c r="I234" t="inlineStr">
         <is>
-          <t>Remove duplicate point records or merge attributes into a single authoritative point.</t>
+          <t>Find duplicate shapes and keep the authoritative record while deleting or merging duplicates.</t>
         </is>
       </c>
       <c r="J234" t="inlineStr">
         <is>
-          <t>ArcGIS Geodatabase Topology Rules</t>
+          <t>QGIS Geometry Checker Plugin</t>
         </is>
       </c>
     </row>
@@ -12796,7 +12788,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>endpoint_unresolved</t>
+          <t>duplicate_geometry_same_layer</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -12806,12 +12798,12 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>evidence_condition</t>
+          <t>data_issue</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
@@ -12826,12 +12818,12 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>A line endpoint could not be classified as a near miss, an orphan, a legitimate terminal or a node-continuation, so the reason it is free is unknown.</t>
+          <t>A feature duplicates the geometry of another feature in the same layer.</t>
         </is>
       </c>
       <c r="I235" t="inlineStr">
         <is>
-          <t>Supply the companion node layer and widen the search radius, then re-triage. An endpoint nobody can explain is not the same as one that is merely tolerated.</t>
+          <t>Review whether duplicate features should be merged, deleted, or linked by shared identifiers.</t>
         </is>
       </c>
       <c r="J235" t="inlineStr"/>
@@ -12844,12 +12836,12 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>epanet_dangling_endpoint</t>
+          <t>duplicate_point</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -12874,15 +12866,19 @@
       </c>
       <c r="H236" t="inlineStr">
         <is>
-          <t>A link names a node that does not exist in the network.</t>
+          <t>Multiple points occupy the same location where duplicates are not allowed.</t>
         </is>
       </c>
       <c r="I236" t="inlineStr">
         <is>
-          <t>Add the missing node or correct the identifier. A dangling endpoint either fails to load or leaves the link unresolved.</t>
-        </is>
-      </c>
-      <c r="J236" t="inlineStr"/>
+          <t>Remove duplicate point records or merge attributes into a single authoritative point.</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>ArcGIS Geodatabase Topology Rules</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -12892,22 +12888,22 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>epanet_disconnected_component</t>
+          <t>endpoint_unresolved</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>data_issue</t>
+          <t>evidence_condition</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
@@ -12922,12 +12918,12 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>Part of the network is not reachable from any supply, so it has no pressure regime and contributes no flow.</t>
+          <t>A line endpoint could not be classified as a near miss, an orphan, a legitimate terminal or a node-continuation, so the reason it is free is unknown.</t>
         </is>
       </c>
       <c r="I237" t="inlineStr">
         <is>
-          <t>Connect the component to the supply or state that it is intentionally isolated, such as a future extension placeholder.</t>
+          <t>Supply the companion node layer and widen the search radius, then re-triage. An endpoint nobody can explain is not the same as one that is merely tolerated.</t>
         </is>
       </c>
       <c r="J237" t="inlineStr"/>
@@ -12940,12 +12936,12 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>epanet_orphaned_node</t>
+          <t>epanet_dangling_endpoint</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>critical</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -12970,12 +12966,12 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>A junction or reservoir is referenced by no link, so it is isolated and contributes no hydraulics.</t>
+          <t>A link names a node that does not exist in the network.</t>
         </is>
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>Connect the node or remove it. Check whether the omission is a truncated export rather than a modelling decision.</t>
+          <t>Add the missing node or correct the identifier. A dangling endpoint either fails to load or leaves the link unresolved.</t>
         </is>
       </c>
       <c r="J238" t="inlineStr"/>
@@ -12988,7 +12984,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>feature_not_split_at_intersection</t>
+          <t>epanet_disconnected_component</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -13018,12 +13014,12 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>A line crosses another feature at an interior point without being split into a network node.</t>
+          <t>Part of the network is not reachable from any supply, so it has no pressure regime and contributes no flow.</t>
         </is>
       </c>
       <c r="I239" t="inlineStr">
         <is>
-          <t>Split the intersecting features at the node or document why the crossing is valid in this network.</t>
+          <t>Connect the component to the supply or state that it is intentionally isolated, such as a future extension placeholder.</t>
         </is>
       </c>
       <c r="J239" t="inlineStr"/>
@@ -13036,7 +13032,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>feature_within_feature</t>
+          <t>epanet_orphaned_node</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -13066,19 +13062,15 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>One feature is completely contained inside another feature of the same layer where that relationship is not expected.</t>
+          <t>A junction or reservoir is referenced by no link, so it is isolated and contributes no hydraulics.</t>
         </is>
       </c>
       <c r="I240" t="inlineStr">
         <is>
-          <t>Review whether containment is legitimate; otherwise split, merge, or delete the nested feature.</t>
-        </is>
-      </c>
-      <c r="J240" t="inlineStr">
-        <is>
-          <t>QGIS Geometry Checker Plugin</t>
-        </is>
-      </c>
+          <t>Connect the node or remove it. Check whether the omission is a truncated export rather than a modelling decision.</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -13088,7 +13080,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>isolated_network_segment</t>
+          <t>feature_not_split_at_intersection</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -13103,7 +13095,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
@@ -13118,12 +13110,12 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>A line segment is isolated from the surrounding network at both endpoints.</t>
+          <t>A line crosses another feature at an interior point without being split into a network node.</t>
         </is>
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>Review whether the segment should connect to nearby infrastructure or be classified as a valid standalone feature.</t>
+          <t>Split the intersecting features at the node or document why the crossing is valid in this network.</t>
         </is>
       </c>
       <c r="J241" t="inlineStr"/>
@@ -13136,7 +13128,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>line_dangle</t>
+          <t>feature_within_feature</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -13151,7 +13143,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -13166,15 +13158,19 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>A line endpoint is dangling where the active profile expects network connectivity.</t>
+          <t>One feature is completely contained inside another feature of the same layer where that relationship is not expected.</t>
         </is>
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>Review endpoint connectivity, service-endpoint rules, and intended network termination behavior.</t>
-        </is>
-      </c>
-      <c r="J242" t="inlineStr"/>
+          <t>Review whether containment is legitimate; otherwise split, merge, or delete the nested feature.</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>QGIS Geometry Checker Plugin</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -13184,24 +13180,24 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>line_has_dangle</t>
+          <t>isolated_network_segment</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>data_issue</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="D243" t="inlineStr">
-        <is>
-          <t>data_issue</t>
-        </is>
-      </c>
-      <c r="E243" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
       <c r="F243" t="inlineStr">
         <is>
           <t>yes</t>
@@ -13214,19 +13210,15 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>A line endpoint is not connected where network continuity is expected.</t>
+          <t>A line segment is isolated from the surrounding network at both endpoints.</t>
         </is>
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>Extend or snap the dangling endpoint to the intended junction if the network should be connected.</t>
-        </is>
-      </c>
-      <c r="J243" t="inlineStr">
-        <is>
-          <t>ArcGIS Geodatabase Topology Rules</t>
-        </is>
-      </c>
+          <t>Review whether the segment should connect to nearby infrastructure or be classified as a valid standalone feature.</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -13236,7 +13228,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>line_has_pseudo_node</t>
+          <t>line_dangle</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -13251,7 +13243,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
@@ -13266,19 +13258,15 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>A line network contains an unnecessary intermediate node that does not represent a true junction.</t>
+          <t>A line endpoint is dangling where the active profile expects network connectivity.</t>
         </is>
       </c>
       <c r="I244" t="inlineStr">
         <is>
-          <t>Merge unnecessarily split line segments where no true junction exists.</t>
-        </is>
-      </c>
-      <c r="J244" t="inlineStr">
-        <is>
-          <t>ArcGIS Geodatabase Topology Rules</t>
-        </is>
-      </c>
+          <t>Review endpoint connectivity, service-endpoint rules, and intended network termination behavior.</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -13288,12 +13276,12 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>line_intersection_same_layer</t>
+          <t>line_has_dangle</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -13318,17 +13306,17 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>Lines in the same layer cross where only endpoint connections are allowed.</t>
+          <t>A line endpoint is not connected where network continuity is expected.</t>
         </is>
       </c>
       <c r="I245" t="inlineStr">
         <is>
-          <t>Split features at valid junctions or correct line placement so only allowed crossings remain.</t>
+          <t>Extend or snap the dangling endpoint to the intended junction if the network should be connected.</t>
         </is>
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>QGIS Topology Checker Plugin</t>
+          <t>ArcGIS Geodatabase Topology Rules</t>
         </is>
       </c>
     </row>
@@ -13340,12 +13328,12 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>narrow_invalid_coverage_gap</t>
+          <t>line_has_pseudo_node</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -13370,17 +13358,17 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>A polygon coverage contains narrow gaps that violate practical edge-matching tolerances even if the gaps are visually subtle. Diagnose with coverage gap checks using a tolerance and clean or snap the coverage to remove slivers.</t>
+          <t>A line network contains an unnecessary intermediate node that does not represent a true junction.</t>
         </is>
       </c>
       <c r="I246" t="inlineStr">
         <is>
-          <t>Use coverage validation and snap/clean tools to close narrow gaps between polygons.</t>
+          <t>Merge unnecessarily split line segments where no true junction exists.</t>
         </is>
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>PostGIS ST_CoverageInvalidEdges</t>
+          <t>ArcGIS Geodatabase Topology Rules</t>
         </is>
       </c>
     </row>
@@ -13392,7 +13380,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>non_edge_matched_polygon_coverage</t>
+          <t>line_intersection_same_layer</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -13422,17 +13410,17 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>Adjacent polygons fail to share identical vertices along common edges, so the set does not form a valid coverage. Diagnose with coverage-validity checks and snap or clean neighboring edges until they match exactly.</t>
+          <t>Lines in the same layer cross where only endpoint connections are allowed.</t>
         </is>
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>Snap shared polygon edges or rebuild the coverage so neighboring polygons share identical boundaries.</t>
+          <t>Split features at valid junctions or correct line placement so only allowed crossings remain.</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>PostGIS ST_CoverageInvalidEdges</t>
+          <t>QGIS Topology Checker Plugin</t>
         </is>
       </c>
     </row>
@@ -13444,12 +13432,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>polygon_gap</t>
+          <t>narrow_invalid_coverage_gap</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -13474,17 +13462,17 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>Voids exist within or between polygons that should create a continuous surface.</t>
+          <t>A polygon coverage contains narrow gaps that violate practical edge-matching tolerances even if the gaps are visually subtle. Diagnose with coverage gap checks using a tolerance and clean or snap the coverage to remove slivers.</t>
         </is>
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>Use topology gap fixes, polygonize workflows, or shared-edge snapping to close uncovered areas.</t>
+          <t>Use coverage validation and snap/clean tools to close narrow gaps between polygons.</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>ArcGIS Geodatabase Topology Rules</t>
+          <t>PostGIS ST_CoverageInvalidEdges</t>
         </is>
       </c>
     </row>
@@ -13496,7 +13484,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>polygon_gap_same_layer</t>
+          <t>non_edge_matched_polygon_coverage</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -13511,7 +13499,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -13526,15 +13514,19 @@
       </c>
       <c r="H249" t="inlineStr">
         <is>
-          <t>An interior gap exists within same-layer polygon coverage.</t>
+          <t>Adjacent polygons fail to share identical vertices along common edges, so the set does not form a valid coverage. Diagnose with coverage-validity checks and snap or clean neighboring edges until they match exactly.</t>
         </is>
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>Review adjacent polygon boundaries and close unintended gaps or document valid voids.</t>
-        </is>
-      </c>
-      <c r="J249" t="inlineStr"/>
+          <t>Snap shared polygon edges or rebuild the coverage so neighboring polygons share identical boundaries.</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>PostGIS ST_CoverageInvalidEdges</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -13544,7 +13536,7 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>polygon_overlap_same_layer</t>
+          <t>polygon_gap</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
@@ -13574,12 +13566,12 @@
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>Polygons in the same feature class overlap when they should form non-overlapping areas.</t>
+          <t>Voids exist within or between polygons that should create a continuous surface.</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>Validate topology and clip or reshape polygons so shared classes no longer overlap.</t>
+          <t>Use topology gap fixes, polygonize workflows, or shared-edge snapping to close uncovered areas.</t>
         </is>
       </c>
       <c r="J250" t="inlineStr">
@@ -13596,7 +13588,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>small_polygon_gap</t>
+          <t>polygon_gap_same_layer</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
@@ -13611,7 +13603,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -13626,19 +13618,15 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>A narrow unintended gap appears between polygons that should share boundaries.</t>
+          <t>An interior gap exists within same-layer polygon coverage.</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>Snap shared edges or use topology validation tools to close narrow gaps.</t>
-        </is>
-      </c>
-      <c r="J251" t="inlineStr">
-        <is>
-          <t>QGIS Geometry Checker Plugin</t>
-        </is>
-      </c>
+          <t>Review adjacent polygon boundaries and close unintended gaps or document valid voids.</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -13648,7 +13636,7 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>small_polygon_overlap</t>
+          <t>polygon_overlap_same_layer</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
@@ -13678,17 +13666,17 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>Adjacent polygons overlap by a small area, often due to snapping or editing errors.</t>
+          <t>Polygons in the same feature class overlap when they should form non-overlapping areas.</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>Use topology fixes, snapping, or edge matching to eliminate overlap slivers between adjacent polygons.</t>
+          <t>Validate topology and clip or reshape polygons so shared classes no longer overlap.</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>QGIS Geometry Checker Plugin</t>
+          <t>ArcGIS Geodatabase Topology Rules</t>
         </is>
       </c>
     </row>
@@ -13700,12 +13688,12 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>suspicious_near_miss_endpoints</t>
+          <t>small_polygon_gap</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -13715,7 +13703,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -13730,15 +13718,19 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>Endpoints are close enough to suggest an unintended near miss but are not snapped together.</t>
+          <t>A narrow unintended gap appears between polygons that should share boundaries.</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>Inspect nearby endpoints and snap them if the separation is unintended or below network tolerance.</t>
-        </is>
-      </c>
-      <c r="J253" t="inlineStr"/>
+          <t>Snap shared edges or use topology validation tools to close narrow gaps.</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>QGIS Geometry Checker Plugin</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -13748,48 +13740,148 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
+          <t>small_polygon_overlap</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>data_issue</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Logical Consistency</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>Adjacent polygons overlap by a small area, often due to snapping or editing errors.</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>Use topology fixes, snapping, or edge matching to eliminate overlap slivers between adjacent polygons.</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>QGIS Geometry Checker Plugin</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>suspicious_near_miss_endpoints</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>data_issue</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>Logical Consistency</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>Endpoints are close enough to suggest an unintended near miss but are not snapped together.</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>Inspect nearby endpoints and snap them if the separation is unintended or below network tolerance.</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>topology</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
           <t>unsnapped_endpoints_within_tolerance</t>
         </is>
       </c>
-      <c r="C254" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="D254" t="inlineStr">
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
         <is>
           <t>data_issue</t>
         </is>
       </c>
-      <c r="E254" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F254" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G254" t="inlineStr">
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
         <is>
           <t>Logical Consistency</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr">
+      <c r="H256" t="inlineStr">
         <is>
           <t>Disconnected endpoints fall within the configured snap tolerance.</t>
         </is>
       </c>
-      <c r="I254" t="inlineStr">
+      <c r="I256" t="inlineStr">
         <is>
           <t>Snap the endpoints or document why the disconnected near match is valid.</t>
         </is>
       </c>
-      <c r="J254" t="inlineStr"/>
+      <c r="J256" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J254"/>
+  <autoFilter ref="A1:J256"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14855,7 +14947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -15098,11 +15190,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>geoqa/cli/__init__.py</t>
+          <t>geoqa/chunking.py</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>422</v>
       </c>
     </row>
     <row r="17">
@@ -15113,7 +15205,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>geoqa/cli/commands/__init__.py</t>
+          <t>geoqa/cli/__init__.py</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -15128,11 +15220,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>geoqa/cli/commands/_common.py</t>
+          <t>geoqa/cli/commands/__init__.py</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>98</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -15143,11 +15235,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>geoqa/cli/commands/audit_archive.py</t>
+          <t>geoqa/cli/commands/_common.py</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20">
@@ -15158,11 +15250,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>geoqa/cli/commands/benchmark.py</t>
+          <t>geoqa/cli/commands/audit_archive.py</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="21">
@@ -15173,11 +15265,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>geoqa/cli/commands/convert.py</t>
+          <t>geoqa/cli/commands/benchmark.py</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>28</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22">
@@ -15188,11 +15280,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>geoqa/cli/commands/profiles.py</t>
+          <t>geoqa/cli/commands/convert.py</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>97</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23">
@@ -15203,11 +15295,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>geoqa/cli/commands/report.py</t>
+          <t>geoqa/cli/commands/profiles.py</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>45</v>
+        <v>97</v>
       </c>
     </row>
     <row r="24">
@@ -15218,11 +15310,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>geoqa/cli/commands/validate.py</t>
+          <t>geoqa/cli/commands/report.py</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>71</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25">
@@ -15233,11 +15325,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>geoqa/cli/main.py</t>
+          <t>geoqa/cli/commands/validate.py</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>34</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26">
@@ -15248,11 +15340,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>geoqa/conversion.py</t>
+          <t>geoqa/cli/main.py</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>490</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27">
@@ -15263,11 +15355,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>geoqa/execution.py</t>
+          <t>geoqa/conversion.py</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>507</v>
+        <v>490</v>
       </c>
     </row>
     <row r="28">
@@ -15278,11 +15370,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>geoqa/expect/__init__.py</t>
+          <t>geoqa/execution.py</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>23</v>
+        <v>507</v>
       </c>
     </row>
     <row r="29">
@@ -15293,11 +15385,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>geoqa/expect/core.py</t>
+          <t>geoqa/expect/__init__.py</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>189</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30">
@@ -15308,11 +15400,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>geoqa/fix/__init__.py</t>
+          <t>geoqa/expect/core.py</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>25</v>
+        <v>189</v>
       </c>
     </row>
     <row r="31">
@@ -15323,11 +15415,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>geoqa/fixes.py</t>
+          <t>geoqa/fix/__init__.py</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>218</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32">
@@ -15338,11 +15430,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>geoqa/gpkg.py</t>
+          <t>geoqa/fixes.py</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>616</v>
+        <v>218</v>
       </c>
     </row>
     <row r="33">
@@ -15353,11 +15445,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>geoqa/hardware.py</t>
+          <t>geoqa/gpkg.py</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>647</v>
+        <v>616</v>
       </c>
     </row>
     <row r="34">
@@ -15368,11 +15460,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>geoqa/hitl.py</t>
+          <t>geoqa/hardware.py</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>435</v>
+        <v>647</v>
       </c>
     </row>
     <row r="35">
@@ -15383,11 +15475,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>geoqa/interactive/__init__.py</t>
+          <t>geoqa/hitl.py</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>5</v>
+        <v>435</v>
       </c>
     </row>
     <row r="36">
@@ -15398,11 +15490,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>geoqa/interactive/validation.py</t>
+          <t>geoqa/interactive/__init__.py</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37">
@@ -15413,11 +15505,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>geoqa/interactive_validation.py</t>
+          <t>geoqa/interactive/validation.py</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>225</v>
+        <v>33</v>
       </c>
     </row>
     <row r="38">
@@ -15428,11 +15520,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>geoqa/packs/__init__.py</t>
+          <t>geoqa/interactive_validation.py</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>37</v>
+        <v>225</v>
       </c>
     </row>
     <row r="39">
@@ -15443,11 +15535,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>geoqa/packs/boundaries/__init__.py</t>
+          <t>geoqa/packs/__init__.py</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>15</v>
+        <v>37</v>
       </c>
     </row>
     <row r="40">
@@ -15458,11 +15550,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>geoqa/packs/boundaries/profile.py</t>
+          <t>geoqa/packs/boundaries/__init__.py</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
     </row>
     <row r="41">
@@ -15473,11 +15565,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>geoqa/packs/boundaries/rules.py</t>
+          <t>geoqa/packs/boundaries/profile.py</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>39</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42">
@@ -15488,11 +15580,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>geoqa/packs/boundaries/thresholds.py</t>
+          <t>geoqa/packs/boundaries/rules.py</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>16</v>
+        <v>39</v>
       </c>
     </row>
     <row r="43">
@@ -15503,11 +15595,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>geoqa/packs/domains.py</t>
+          <t>geoqa/packs/boundaries/thresholds.py</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>327</v>
+        <v>16</v>
       </c>
     </row>
     <row r="44">
@@ -15518,11 +15610,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>geoqa/packs/land_use/__init__.py</t>
+          <t>geoqa/packs/domains.py</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>15</v>
+        <v>327</v>
       </c>
     </row>
     <row r="45">
@@ -15533,11 +15625,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>geoqa/packs/land_use/profile.py</t>
+          <t>geoqa/packs/land_use/__init__.py</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>93</v>
+        <v>15</v>
       </c>
     </row>
     <row r="46">
@@ -15548,11 +15640,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>geoqa/packs/land_use/rules.py</t>
+          <t>geoqa/packs/land_use/profile.py</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>25</v>
+        <v>93</v>
       </c>
     </row>
     <row r="47">
@@ -15563,11 +15655,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>geoqa/packs/land_use/thresholds.py</t>
+          <t>geoqa/packs/land_use/rules.py</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="48">
@@ -15578,11 +15670,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>geoqa/packs/water_network/__init__.py</t>
+          <t>geoqa/packs/land_use/thresholds.py</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="49">
@@ -15593,11 +15685,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>geoqa/packs/water_network/profile.py</t>
+          <t>geoqa/packs/water_network/__init__.py</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>119</v>
+        <v>23</v>
       </c>
     </row>
     <row r="50">
@@ -15608,11 +15700,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>geoqa/packs/water_network/rules.py</t>
+          <t>geoqa/packs/water_network/profile.py</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>294</v>
+        <v>119</v>
       </c>
     </row>
     <row r="51">
@@ -15623,11 +15715,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>geoqa/packs/water_network/schema.py</t>
+          <t>geoqa/packs/water_network/rules.py</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>73</v>
+        <v>294</v>
       </c>
     </row>
     <row r="52">
@@ -15638,11 +15730,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>geoqa/packs/water_network/thresholds.py</t>
+          <t>geoqa/packs/water_network/schema.py</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>46</v>
+        <v>73</v>
       </c>
     </row>
     <row r="53">
@@ -15653,11 +15745,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>geoqa/plugins/__init__.py</t>
+          <t>geoqa/packs/water_network/thresholds.py</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>6</v>
+        <v>46</v>
       </c>
     </row>
     <row r="54">
@@ -15668,11 +15760,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>geoqa/plugins/base.py</t>
+          <t>geoqa/plugins/__init__.py</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>37</v>
+        <v>6</v>
       </c>
     </row>
     <row r="55">
@@ -15683,11 +15775,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>geoqa/plugins/dma/__init__.py</t>
+          <t>geoqa/plugins/base.py</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
     </row>
     <row r="56">
@@ -15698,11 +15790,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>geoqa/plugins/dma/common.py</t>
+          <t>geoqa/plugins/dma/__init__.py</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>198</v>
+        <v>25</v>
       </c>
     </row>
     <row r="57">
@@ -15713,11 +15805,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>geoqa/plugins/dma/dma_cross_name_nested.py</t>
+          <t>geoqa/plugins/dma/common.py</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>113</v>
+        <v>198</v>
       </c>
     </row>
     <row r="58">
@@ -15728,11 +15820,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>geoqa/plugins/dma/dma_multipart_polygons.py</t>
+          <t>geoqa/plugins/dma/dma_cross_name_nested.py</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>74</v>
+        <v>113</v>
       </c>
     </row>
     <row r="59">
@@ -15743,11 +15835,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>geoqa/plugins/dma/dma_overlap_conflicts.py</t>
+          <t>geoqa/plugins/dma/dma_multipart_polygons.py</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="60">
@@ -15758,11 +15850,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>geoqa/plugins/dma/dma_same_name_nested.py</t>
+          <t>geoqa/plugins/dma/dma_overlap_conflicts.py</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>119</v>
+        <v>81</v>
       </c>
     </row>
     <row r="61">
@@ -15773,11 +15865,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>geoqa/plugins/registry.py</t>
+          <t>geoqa/plugins/dma/dma_same_name_nested.py</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>38</v>
+        <v>119</v>
       </c>
     </row>
     <row r="62">
@@ -15788,11 +15880,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>geoqa/problem_registry.py</t>
+          <t>geoqa/plugins/registry.py</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1824</v>
+        <v>38</v>
       </c>
     </row>
     <row r="63">
@@ -15803,11 +15895,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>geoqa/profile_registry.py</t>
+          <t>geoqa/problem_registry.py</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>275</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="64">
@@ -15818,11 +15910,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>geoqa/proj_env.py</t>
+          <t>geoqa/profile_registry.py</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>116</v>
+        <v>275</v>
       </c>
     </row>
     <row r="65">
@@ -15833,11 +15925,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>geoqa/qgis_export.py</t>
+          <t>geoqa/proj_env.py</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>90</v>
+        <v>116</v>
       </c>
     </row>
     <row r="66">
@@ -15848,11 +15940,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>geoqa/qgis_integration.py</t>
+          <t>geoqa/qgis_export.py</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>376</v>
+        <v>90</v>
       </c>
     </row>
     <row r="67">
@@ -15863,11 +15955,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>geoqa/runner.py</t>
+          <t>geoqa/qgis_integration.py</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>65</v>
+        <v>376</v>
       </c>
     </row>
     <row r="68">
@@ -15878,11 +15970,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>geoqa/script_base.py</t>
+          <t>geoqa/runner.py</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>77</v>
+        <v>65</v>
       </c>
     </row>
     <row r="69">
@@ -15893,11 +15985,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>geoqa/serialization/__init__.py</t>
+          <t>geoqa/script_base.py</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>5</v>
+        <v>77</v>
       </c>
     </row>
     <row r="70">
@@ -15908,11 +16000,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>geoqa/thermal.py</t>
+          <t>geoqa/serialization/__init__.py</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>413</v>
+        <v>5</v>
       </c>
     </row>
     <row r="71">
@@ -15923,26 +16015,26 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>geoqa/validation_runtime.py</t>
+          <t>geoqa/thermal.py</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2010</v>
+        <v>413</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>reports</t>
+          <t>other</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>geoqa/reports/__init__.py</t>
+          <t>geoqa/validation_runtime.py</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>5</v>
+        <v>2010</v>
       </c>
     </row>
     <row r="73">
@@ -15953,11 +16045,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>geoqa/reports/aggregation.py</t>
+          <t>geoqa/reports/__init__.py</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>414</v>
+        <v>5</v>
       </c>
     </row>
     <row r="74">
@@ -15968,11 +16060,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>geoqa/reports/explanations.py</t>
+          <t>geoqa/reports/aggregation.py</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>65</v>
+        <v>414</v>
       </c>
     </row>
     <row r="75">
@@ -15983,26 +16075,26 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>geoqa/reports/report_generator.py</t>
+          <t>geoqa/reports/explanations.py</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>308</v>
+        <v>65</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>validators</t>
+          <t>reports</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>geoqa/validations/__init__.py</t>
+          <t>geoqa/reports/report_generator.py</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>39</v>
+        <v>308</v>
       </c>
     </row>
     <row r="77">
@@ -16013,11 +16105,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>geoqa/validations/accuracy.py</t>
+          <t>geoqa/validations/__init__.py</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>239</v>
+        <v>39</v>
       </c>
     </row>
     <row r="78">
@@ -16028,11 +16120,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>geoqa/validations/archive.py</t>
+          <t>geoqa/validations/accuracy.py</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>761</v>
+        <v>239</v>
       </c>
     </row>
     <row r="79">
@@ -16043,11 +16135,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>geoqa/validations/attributes.py</t>
+          <t>geoqa/validations/archive.py</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>128</v>
+        <v>761</v>
       </c>
     </row>
     <row r="80">
@@ -16058,11 +16150,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>geoqa/validations/axis_order.py</t>
+          <t>geoqa/validations/attributes.py</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>592</v>
+        <v>128</v>
       </c>
     </row>
     <row r="81">
@@ -16073,11 +16165,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>geoqa/validations/base.py</t>
+          <t>geoqa/validations/axis_order.py</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>225</v>
+        <v>592</v>
       </c>
     </row>
     <row r="82">
@@ -16088,11 +16180,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>geoqa/validations/boundary_conformance.py</t>
+          <t>geoqa/validations/base.py</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>569</v>
+        <v>225</v>
       </c>
     </row>
     <row r="83">
@@ -16103,11 +16195,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>geoqa/validations/clip.py</t>
+          <t>geoqa/validations/boundary_conformance.py</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>515</v>
+        <v>569</v>
       </c>
     </row>
     <row r="84">
@@ -16118,11 +16210,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>geoqa/validations/cog.py</t>
+          <t>geoqa/validations/clip.py</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>299</v>
+        <v>515</v>
       </c>
     </row>
     <row r="85">
@@ -16133,11 +16225,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>geoqa/validations/credentials.py</t>
+          <t>geoqa/validations/cog.py</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>441</v>
+        <v>299</v>
       </c>
     </row>
     <row r="86">
@@ -16148,11 +16240,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>geoqa/validations/crs.py</t>
+          <t>geoqa/validations/credentials.py</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>94</v>
+        <v>441</v>
       </c>
     </row>
     <row r="87">
@@ -16163,11 +16255,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>geoqa/validations/crs_units.py</t>
+          <t>geoqa/validations/crs.py</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>639</v>
+        <v>94</v>
       </c>
     </row>
     <row r="88">
@@ -16178,11 +16270,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>geoqa/validations/dimension.py</t>
+          <t>geoqa/validations/crs_units.py</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>300</v>
+        <v>639</v>
       </c>
     </row>
     <row r="89">
@@ -16193,11 +16285,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>geoqa/validations/endpoint_triage.py</t>
+          <t>geoqa/validations/dimension.py</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>723</v>
+        <v>300</v>
       </c>
     </row>
     <row r="90">
@@ -16208,11 +16300,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>geoqa/validations/epanet.py</t>
+          <t>geoqa/validations/endpoint_triage.py</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>756</v>
+        <v>723</v>
       </c>
     </row>
     <row r="91">
@@ -16223,11 +16315,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>geoqa/validations/geometry.py</t>
+          <t>geoqa/validations/epanet.py</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>258</v>
+        <v>756</v>
       </c>
     </row>
     <row r="92">
@@ -16238,11 +16330,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>geoqa/validations/governance.py</t>
+          <t>geoqa/validations/geometry.py</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>396</v>
+        <v>258</v>
       </c>
     </row>
     <row r="93">
@@ -16253,11 +16345,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>geoqa/validations/hyperspectral.py</t>
+          <t>geoqa/validations/governance.py</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>769</v>
+        <v>396</v>
       </c>
     </row>
     <row r="94">
@@ -16268,11 +16360,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>geoqa/validations/integrity.py</t>
+          <t>geoqa/validations/hyperspectral.py</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>98</v>
+        <v>769</v>
       </c>
     </row>
     <row r="95">
@@ -16283,11 +16375,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>geoqa/validations/metadata.py</t>
+          <t>geoqa/validations/integrity.py</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>60</v>
+        <v>98</v>
       </c>
     </row>
     <row r="96">
@@ -16298,11 +16390,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>geoqa/validations/metric_constants.py</t>
+          <t>geoqa/validations/metadata.py</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>335</v>
+        <v>60</v>
       </c>
     </row>
     <row r="97">
@@ -16313,11 +16405,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>geoqa/validations/night_flow.py</t>
+          <t>geoqa/validations/metric_constants.py</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>502</v>
+        <v>335</v>
       </c>
     </row>
     <row r="98">
@@ -16328,11 +16420,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>geoqa/validations/osm.py</t>
+          <t>geoqa/validations/night_flow.py</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>330</v>
+        <v>502</v>
       </c>
     </row>
     <row r="99">
@@ -16343,11 +16435,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>geoqa/validations/payload_columns.py</t>
+          <t>geoqa/validations/osm.py</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>248</v>
+        <v>330</v>
       </c>
     </row>
     <row r="100">
@@ -16358,11 +16450,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>geoqa/validations/raster.py</t>
+          <t>geoqa/validations/payload_columns.py</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>507</v>
+        <v>248</v>
       </c>
     </row>
     <row r="101">
@@ -16373,11 +16465,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>geoqa/validations/reference_cases.py</t>
+          <t>geoqa/validations/raster.py</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="102">
@@ -16388,11 +16480,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>geoqa/validations/repeat_incident.py</t>
+          <t>geoqa/validations/reference_cases.py</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>430</v>
+        <v>505</v>
       </c>
     </row>
     <row r="103">
@@ -16403,11 +16495,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>geoqa/validations/spectral.py</t>
+          <t>geoqa/validations/repeat_incident.py</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>280</v>
+        <v>430</v>
       </c>
     </row>
     <row r="104">
@@ -16418,11 +16510,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>geoqa/validations/tabular.py</t>
+          <t>geoqa/validations/spectral.py</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>687</v>
+        <v>280</v>
       </c>
     </row>
     <row r="105">
@@ -16433,11 +16525,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>geoqa/validations/topology.py</t>
+          <t>geoqa/validations/tabular.py</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>962</v>
+        <v>687</v>
       </c>
     </row>
     <row r="106">
@@ -16448,11 +16540,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>geoqa/validations/vertical_datum.py</t>
+          <t>geoqa/validations/topology.py</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>432</v>
+        <v>962</v>
       </c>
     </row>
     <row r="107">
@@ -16463,11 +16555,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>geoqa/validations/water_balance.py</t>
+          <t>geoqa/validations/vertical_datum.py</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>456</v>
+        <v>432</v>
       </c>
     </row>
     <row r="108">
@@ -16478,11 +16570,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>geoqa/validations/water_loss.py</t>
+          <t>geoqa/validations/water_balance.py</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>441</v>
+        <v>456</v>
       </c>
     </row>
     <row r="109">
@@ -16493,15 +16585,30 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
+          <t>geoqa/validations/water_loss.py</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>validators</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
           <t>geoqa/validations/workbook_media.py</t>
         </is>
       </c>
-      <c r="C109" t="n">
+      <c r="C110" t="n">
         <v>526</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C109"/>
+  <autoFilter ref="A1:C110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>